<commit_message>
Add risk assessment to ITS project dashboard
</commit_message>
<xml_diff>
--- a/ITS Project Tracking/ITS_Project_Tracking_Public_2026-09-24.xlsx
+++ b/ITS Project Tracking/ITS_Project_Tracking_Public_2026-09-24.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Projects'!$A$1:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Projects'!$A$1:$N$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="mmm d, yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mmm d, yyyy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -70,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -81,7 +80,7 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -90,7 +89,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -493,7 +498,9 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="31" customWidth="1" min="10" max="10"/>
     <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -552,7 +559,17 @@
           <t>project_type</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>risk_level</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>risk_category</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>milestones_completed</t>
         </is>
@@ -587,7 +604,7 @@
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="8" t="n">
         <v>46660</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -610,7 +627,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -641,7 +668,7 @@
       <c r="F3" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="9" t="n">
         <v>46387</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -664,7 +691,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -695,7 +732,7 @@
       <c r="F4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="8" t="n">
         <v>46568</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -718,7 +755,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Priority or Resourcing</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -749,7 +796,7 @@
       <c r="F5" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="9" t="n">
         <v>46568</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -772,7 +819,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>External Dependency</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -803,7 +860,7 @@
       <c r="F6" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="8" t="n">
         <v>46568</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -826,7 +883,17 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Priority or Resourcing</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -857,7 +924,7 @@
       <c r="F7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="9" t="n">
         <v>46477</v>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -880,7 +947,17 @@
           <t>Compliance or Mandated</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Priority or Resourcing</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -911,7 +988,7 @@
       <c r="F8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="8" t="n">
         <v>46568</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -934,7 +1011,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -965,7 +1052,7 @@
       <c r="F9" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="9" t="n">
         <v>46387</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -988,7 +1075,17 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1019,7 +1116,7 @@
       <c r="F10" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="8" t="n">
         <v>46418</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1042,7 +1139,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1073,7 +1180,7 @@
       <c r="F11" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1096,7 +1203,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1127,7 +1244,7 @@
       <c r="F12" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="8" t="n">
         <v>46477</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1150,7 +1267,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1181,7 +1308,7 @@
       <c r="F13" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1204,7 +1331,17 @@
           <t>Compliance or Mandated</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Regulatory Deadline</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1235,7 +1372,7 @@
       <c r="F14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="8" t="n">
         <v>46538</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1258,7 +1395,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1289,7 +1436,7 @@
       <c r="F15" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="9" t="n">
         <v>46387</v>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1312,7 +1459,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1343,7 +1500,7 @@
       <c r="F16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="8" t="n">
         <v>46752</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1366,7 +1523,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1397,7 +1564,7 @@
       <c r="F17" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="9" t="n">
         <v>46385</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1420,7 +1587,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Not Reported</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1451,7 +1628,7 @@
       <c r="F18" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="G18" s="8" t="n">
         <v>46418</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1474,7 +1651,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>EMS migration completed</t>
         </is>
@@ -1509,7 +1696,7 @@
       <c r="F19" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="9" t="n">
         <v>46387</v>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1532,7 +1719,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>External Dependency</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1563,7 +1760,7 @@
       <c r="F20" s="3" t="n">
         <v>85</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="8" t="n">
         <v>46326</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1586,7 +1783,17 @@
           <t>Innovation or Pilot</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Pilot nearing completion</t>
         </is>
@@ -1621,7 +1828,7 @@
       <c r="F21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1644,7 +1851,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1675,7 +1892,7 @@
       <c r="F22" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="G22" s="8" t="n">
         <v>46507</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1698,7 +1915,17 @@
           <t>Compliance or Mandated</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1729,7 +1956,7 @@
       <c r="F23" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="9" t="n">
         <v>46446</v>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1752,7 +1979,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1783,7 +2020,7 @@
       <c r="F24" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="G24" s="8" t="n">
         <v>46387</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1806,7 +2043,17 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1837,7 +2084,7 @@
       <c r="F25" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="G25" s="7" t="n">
+      <c r="G25" s="9" t="n">
         <v>46477</v>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -1860,7 +2107,17 @@
           <t>Modernization or Upgrade</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1891,7 +2148,7 @@
       <c r="F26" s="3" t="n">
         <v>79</v>
       </c>
-      <c r="G26" s="4" t="n"/>
+      <c r="G26" s="8" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1908,7 +2165,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1939,7 +2206,7 @@
       <c r="F27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="7" t="n">
+      <c r="G27" s="9" t="n">
         <v>46568</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -1962,7 +2229,17 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1993,7 +2270,7 @@
       <c r="F28" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="4" t="n">
+      <c r="G28" s="8" t="n">
         <v>46387</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2016,7 +2293,17 @@
           <t>New Capability</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>External Dependency</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2047,7 +2334,7 @@
       <c r="F29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="7" t="n">
+      <c r="G29" s="9" t="n">
         <v>46418</v>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2070,10 +2357,20 @@
           <t>Innovation or Pilot</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>None Reported</t>
+        </is>
+      </c>
+      <c r="N29" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A1:N29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>